<commit_message>
data: update review_products.xlsx with first batch of 4 funny/novelty products
</commit_message>
<xml_diff>
--- a/review_products.xlsx
+++ b/review_products.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -521,41 +521,10 @@
       </c>
     </row>
     <row r="2" ht="39.95" customHeight="1">
-      <c r="A2" s="2" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>วางรายละเอียดสินค้าจาก Shopee ทั้งหมดที่นี่</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/xxx</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>https://s.lazada.co.th/xxx</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://down-th.img.susercontent.com/xxx.jpg</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>ลด 20%</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="345" customHeight="1">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>RAY-BAN JUSTIN- RB4165F 601/71
 Ray-Ban เรแบนเป็นผู้นำด้านการผลิตแว่นกันแดด และแว่นสายตา ที่ได้ความนิยมมากที่สุดทั่วโลก มีให้เลือกหลากหลายสไตล์ เหมาะกับทุกคน และใส่ได้ทั้งผู้หญิงและผู้ชาย
@@ -569,23 +538,23 @@
 Lens Material: Polycarbonate Standard</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>https://s.shopee.co.th/AUqz80oxUd</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>https://s.lazada.co.th/s.Z6PzJE?c=b&amp;t=p-ijr1Q-svKWG</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>https://down-th.img.susercontent.com/file/th-11134201-7r990-lscec08f21gm73.webp
 https://down-th.img.susercontent.com/file/th-11134201-7r98y-lscec0amysmu78.webp</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">฿5,130
 final price indicator icon
@@ -597,17 +566,17 @@
 </t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>done 2026-05-21 13:15</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="409.5" customHeight="1">
-      <c r="A4" t="n">
+    <row r="3" ht="345" customHeight="1">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Sony BRAVIA 3 ทีวี 55 นิ้ว รุ่น K-55S30 4K Ultra HD Smart TV (Google TV) | 4K HDR Processor X1
 รายละเอียดสินค้า
@@ -627,22 +596,22 @@
 เรียกดูภาพยนตร์และรายการทีวีมากกว่า 400,000 ตอนจากบริการสตรีมมิ่งของคุณทั้งหมดในที่เดียว โดยจัดเป็นหัวข้อและแนวเนื้อหาไว้ตามสิ่งที่คุณสนใจ</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>https://s.shopee.co.th/10zvLKc6Ji</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>https://s.lazada.co.th/s.Z6mEyG?c=a&amp;t=p-i0-s0&amp;sub_id1=W1</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>https://down-th.img.susercontent.com/file/th-11134207-7r98v-lvsn9yh5vql9c5.webp</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">฿20,500
 final price indicator icon
@@ -650,6 +619,110 @@
 โค้ดส่วนลดร้านค้า
 ลด ฿1.99k
 </t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="409.5" customHeight="1">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ความแปลกใหม่ฟุตบอลซิลิโคนไฟกลางคืนชาร์จโคมไฟกลางคืนนอนพร้อมหรี่แสงได้ 3 ระดับเนอสเซอรี่ข้างเตียงสัมผัสโคมไฟสําหรับตกแต่งห้อง</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3B4Y0E5z3a</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/sg-11134201-824jf-me523nns7q4g2a.webp</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ลด 32% เหลือ ฿359 (ปกติ ฿527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CODเครื่องลอกเปลือกองุ่นไฟฟ้าอัตโนมัติ เครื่องลอกเปลือกผลไม้โดยไม่ต้องใช้มือ เครื่องเตรียมผลไม้ ช่วยประหยัดแรง</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/902Kx1OzPK</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/sg-11134201-82593-mgc0wefye8eg8f.webp</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ราคาหลังโค้ดส่วนลด ฿256</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Aimi ชุดกันฝน ชุดกันน้ำ เสื้อกันฝน มีแถบสะท้อนแสง รุ่นหมวกติดเสื้อ คุณภาพดีราคาถูกมีหลายสีให้เลือก</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4Ax5GMKOTb</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/th-11134207-81ztm-mnjwc17ne13541.webp</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ราคาหลังโค้ดส่วนลด ฿129</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sony BRAVIA 3 ทีวี 55 นิ้ว รุ่น K-55S30 4K Ultra HD Smart TV (Google TV) | 4K HDR Processor X1™</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/5L92hVfwWK</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/th-11134207-81zte-mojth82buz2l9f.webp</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ราคาหลังโค้ดส่วนลด ฿20,500</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(kram): enforce 3rd-party curator persona, 2-sided decision questions, add 40 fresh products, and update review log
</commit_message>
<xml_diff>
--- a/review_products.xlsx
+++ b/review_products.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="630" yWindow="615" windowWidth="37095" windowHeight="17310" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="posted_state" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="posted_state" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G177"/>
+  <dimension ref="A1:G217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5200,6 +5200,1006 @@
       <c r="G177" t="inlineStr">
         <is>
           <t>done 2026-08-03 20:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>91</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>ถุงสูญญากาศ เก็บเสื้อผ้าผ้าห่มผ้านวมจัดเก็บของกระชับพื้นที่แพ็คของเดินทางถุงใส่เสื้อผ้าพกพา ราคาต่อชิ้น(แบบใส)</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9AMxjrqLKA</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-7rasc-m0pot616b6pmd7.webp</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>฿10.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>92</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Goody Home ชั้นวางของแบบวางตั้ง ออกแบบให้ระบายน้ำด้านล่างได้ วางของใช้ในพื้นที่ที่โดนน้ำได้</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/111G0rV7s3</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-7r98t-m03zneg13id66d.webp</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>฿65.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>93</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Deli ถุงคลุมเสื้อผ้า ถุงใส่สูท ที่คลุมเสื้อผ้า มีซิปด้านหน้า หลายขนาด ป้องกันฝุ่น Clothing Dust Bag</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1gGwo5adCO</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztf-mgw2ykjq12by14.webp</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>฿26.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>94</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Deli ถุงสูญญากาศ 1ใบ มีวาล์ว ถุงเก็บผ้านวม จัดเก็บผ้านวม ประหยัดพื้นที่ สามารถใช้งานซ้ำ Vacuum Bag</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3B5kaqdeSH</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztn-mgw2x8mi3zewbe.webp</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>฿17.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>95</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>ถุงคลุมเสื้อผ้า(หนาพิเศษ2ชั้น)กันฝุ่น กันยับแบบมีซิป 4ขนาด ถุงใส่สูท ถุงใส่เสื้อผ้า ที่คลุมเสื้อผ้า Clothing Dust Bag</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1gGwo5sA40</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/sg-11134201-825zq-mlq2ylhwts7779.webp</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>฿21.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>96</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>ใหม่❗ถุงสูญญากาศ จัดเก็บเสื้อผ้า&amp;ผ้านวม ถุงประหยัดพื้นที่ ถุงสูญญากาศมีวาล์วซิปล็อค2ชั้น หนาพิเศษใช้ซ้ำได้(ราคาต่อ1ใบ)</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7KvJYVbXRq</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-7qul6-li126pfagwwz75.webp</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>฿11.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>97</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>🐻💖ถุงสูญญากาศ จัดเก็บผ้านวม ถุงสูญญากาศประหยัดพื้นที่ มีจุกวาล์ว(ราคา1ใบ)💖🐻</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9zw4jPZUyo</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-7qul4-ljqfd50uri2x8e.webp</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>฿10.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>98</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>🥳ถุงสูญญากาศ จัดเก็บเสื้อผ้าผ้านวมเป็นระเบียบ ถุงเก็บผ้านวมมีจุกวาวล์ซิปล็อค2ชั้น ถุงประหยัดพื้นที่จัดเก็บ ลายแบร์บริค🥳</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4fuYNc3DjC</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-7ras8-m0poxd0fdcrc2f.webp</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>฿11.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>99</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>ถุงสูญญากาศ 1ใบ มีวาล์ว ถุงเก็บผ้านวม ถุงสุญญากาศ จัดเก็บผ้านวม ประหยัดพื้นที่ สามารถใช้งานซ้ำ Storage Vacuum Bag</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1VxWbnO4iR</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-7r98t-lxw9judbmo4w4f.webp</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>฿9.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>100</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>ที่วางแก้ว แบบหนีบโต๊ะ ปรับ 3 ระดับ หมุน 360 องศา ประหยัดพื้นที่ เก็บซ่อนใต้โต๊ะ ติดตั้งง่าย พร้อมส่งในไทย!</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/80B0Lk7r2g</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztj-mplnq6kpx4wba6.webp</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>฿97.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>101</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>ขวดแก้วใส่เครื่องปรุงอาหารพร้อมช้อนตักในตัว ใช้งานง่าย สะดวก จัดเก็บเป็นระเบียบ</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/5fn5ZSKnFY</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-7rasj-ma8ady0pgs5v65.webp</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>฿14.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>102</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>【มาพร้อมกับ 12 หน้า】สมุดเก็บเอกสาร、แฟ้มจัดเก็บขนาดใหญ่ ที่จัดระเบียบเอกสารครอบครัวหนังหนาพรีเมี่ยมพร้อมกระเป๋าซีลด้านข้างหลายขนาด (A4/B5) หน้าโปร่งใสกันฝุ่นและความชื้นเหมาะสําหรับใบรับรองและไฟล์ส</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9pceX7EHSS</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/cn-11134207-820l4-micqznfxojy955.webp</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>฿69.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>103</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>【จัดส่งที่รวดเร็ว】แผ่นปา DIY แผ่นรูพลาสติกสำหรับจัดเก็บบนโต๊ะพร้อมชุดติดตั้ง ตัวจัดระเบียบโต๊ะเล่นเกม</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8KnqkMSrKP</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztn-mlbudatj51xg78.webp</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>฿43.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>104</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Deli ถุงสูญญากาศ ถุงสูญญากาศจัดเก็บของ มีวาล์ว ประหยัดพื้นที่ ใช้งานซ้ำได้ Storage Vacuum Bag</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7VEjkpaMXa</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztp-mefkkjk10irkb8.webp</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>฿18.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>105</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Aimilo ไม้แขวนเสื้อ 8 ตะขอ กันลื่น ประหยัดพื้นที่ ที่เก็บเสื้อผ้า ไม้แขวนผ้าอเนกประสงค์ แขวนสายเดี่ยว/บรา/เข็มขัด</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/5LAFAqsRR4</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81zto-mp7ec1i114wfab.webp</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>฿16.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>106</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>noordic ชั้นวางของบนโต๊ะ ชั้นเก็บของ 2ชั้น ประหยัดพื้นที่ชั้นวางเดสก์ท็อป ชั้นอเนกประสงค์ สีขาวA1</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/2qSuCGAl4V</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-7rasd-mas1qf3l0nxye7.webp</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>฿67.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>107</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>ชั้นเก็บผ้า ลายแพนด้า ที่เก็บถุงเท้า ชุดชั้นใน สามชั้น ถุงเก็บของ ใส่เสื้อผ้า เก็บผ้า ถุงเก็บผ้า เก็บกระเป๋า</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/2LWdbLKhlZ</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81zte-mfnhf8gv711kae.webp</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>฿36.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>108</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>ชั้นวางรองเท้า ปรับได้3ระดับ ประหยัดพื้นที่ ที่เก็บรองเท้า อุปกรณ์เก็บรองเท้าพลาสติก พับเก็บได้ ที่จัดระเบียบรองเท้า</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/30mKOZMI9J</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/sg-11134201-7rfgd-m3mzspb77207ff.webp</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>฿8.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>109</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>🔥【INS สไตล์】ชั้นวางของบนโต๊ะ ชั้นจัดระเบียบบนโต๊ะทำงาน ชั้นวางอเนกประสงค์ ชั้นวางของ ประหยัดพื้นที่ ติดตั้งง่าย</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1Le6PVbVMF</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztq-mitxca7ji80097.webp</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>฿89.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>110</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>กระเป๋าเคลื่อนย้ายความจุขนาดใหญ่ 110ล/180ล/240ล กันน้ําและกันฝุ่นที่ทนทาน เหมาะสําหรับใส่เสื้อผ้าและเครื่องนอน</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9pceX8DX6K</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/cn-11134207-820l4-mj50iw22nton7d.webp</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>฿48.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>111</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>ผ้าเช็ดกระจกไมโครไฟเบอร์-กระจกอัตโนมัติ ไร้ร่องรอย เช็ด-หนาซุปเปอร์ดูดซับน้ํานํามาใช้ใหม่-ครัวเรือนล้างจานเศษผ้า-ผ้าขนหนูล้างรถมายากล-</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/18iobxFlh</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/sg-11134201-7rdyg-lyasiiofhnvs5f.webp</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>฿5.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>112</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>LOGESKI น้ำยาล้างห้องน้ำ ล้างชักโครก ไม่ต้องขัด ขจัดคราบหนัก ตะกรัน คราบเหลือง ดับกลิ่น ฆ่าเชื้อ 99%</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9AMxjSRWEV</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/cn-11134207-820l4-mq5ye0zrpf676a.webp</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>฿101.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>113</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>LOGESKI น้ำยาล้างเครื่องซักผ้า ไม่ต้องแช่ ขจัดคราบฝังแน่น ลดกลิ่นอับ ฆ่าเชื้อ 99.9%</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8V7GwEd8CN</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/cn-11134207-7ras8-mao08sgtxeb04e.webp</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>฿86.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>114</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>LOGESKI น้ำยาล้างห้องน้ำ โฟมทำความสะอาด ไม่ต้องขัด สลายคราบตะกรัน เชื้อรา คราบเหลือง ดับกลิ่น</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/18iocHsRA</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/cn-11134207-820l4-mji9ddjg6neufd.webp</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>฿222.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>115</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>ผ้าไมโครไฟเบอร์ 3D ขนาด 400แกรม 25X25CM เกรดพรีเมี่ยม หนานุ่ม ซับน้ำไว ทำความสะอาดอเนกประสงค์</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/2g9TzWGf7E</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztn-mnfgv5sgi7t035.webp</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>฿4.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>116</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>[ซื้อ 4 แถม 1/3 ถุง ]ผ้าเปียกทำความสะอาดครัว Kiss Aimy กลิ่นเลมอน ขจัดครา</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/6pz2xB5CTI</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztj-mpf2wiqngidofd.webp</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>฿189.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>117</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Yotex เครื่องปั่นอาหารเด็ก เครื่องปั่นกระเทียม เครื่องปั่น การทำงานด้วยปุ่มเดียว เครื่องปั่นพริก 1000ML ทำความสะอาดง่าย</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/2LWdauWmR2</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81zth-mhtuyubih9fn04.webp</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>฿151.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>118</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>(ร้านนี้ส่งไว+ผงข้นฟรี )ไอ-โชว์ หัวเชื้อน้ำยาล้างจานสูตรเข้มข้น ขจัดคราบมัน 8 สูตร 8กลิ่น 400มิล</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7VEjkPKGDm</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-7rasd-m6qcrl032w1hc1.webp</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>฿21.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>119</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>BOOMJOY แปรงทําความสะอาดฝักบัวและชุดขัดอ่างอาบน้ํา ด้ามยาว 58 ซม. พร้อมแผ่นใยขัด 2 แผ่น และแผ่นไมโครไฟเบอร์ 1 แผ่น สีเทา</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7pra91RRnU</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/cn-11134207-7ras8-m3q4rmtmlq2yde.webp</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>฿335.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>120</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Rabito ผลิตภัณฑ์ทำความสะอาดสเปรย์ทำความสะอาดสำหรับผ้า พรม เบาะรถ โซฟา ไม่ต้องใช้น้ำ Cleaning ไม่ต้องเมื่อยขยี้ ไม่ระคายเ</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8V7GwFXunQ</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81zto-mn0veu8izdac3f.webp</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>฿109.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>121</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>ROJUKISS Deep Cleansing Micellar Water 400ml โรจูคิส ไมเซล่าวอเตอร์ ทำความสะอาดผิวล้ำลึก สลายเมคอัพ อ่อนโยนต่อผิว</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7AbtLni0eu</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/sg-11134201-8259w-mqja2tfrz95af7.webp</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>฿129.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>122</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>ผ้าไมโครไฟเบอร์ 3D ขนาด 400แกรม 30X30 CM เกรดพรีเมี่ยม หนานุ่ม ซับน้ำไว ทำความสะอาดอเนกประสงค์</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7pra91oGrE</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztf-mnfgx95jxret4b.webp</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>฿6.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>123</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>ฟองน้ําไมโครไฟเบอร์ทําความสะอาดอเนกประสงค์</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/111G0TMKPR</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztq-mhzqlbjyyfb63e.webp</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>฿5.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>124</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>ถังปั่นไม้ม๊อบ ถังปั่นไม้ถูพื้น Spin Mop ชุดถังปั่นพลาสติก ชุดทำความสะอาดพื้น ไม้ถูพื้น ไม้ม๊อบ ผ้าม๊อบไมโครไฟเบอร์.</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7fY9wj6EHF</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-7rasi-m3bulq72u31ka1.webp</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>฿96.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>125</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>HOMESTIC ไม้ถูพร้อมถังปั่น ตัวถัง 2 ระบบ ซักทำความสะอาดและปั่นแห้ง ชุดถังปั่นสแตนเลส + ไม้ถูพื้น</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9pceWi8Dx7</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztf-mn14s1xi0o3n65.webp</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>฿95.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>126</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>【5KG】Botare ผลิตภัณฑ์ซักผ้ากลิ่นทับทิม หอมยาวนาน ทำความสะอาดล้ำลึก 1ขวด 5000ml</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8pk7KsIuCh</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztl-mo3epycylw5c5e.webp</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>฿135.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>127</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>(ซื้อ 3 แถม 2 รวม 400 แผ่น) แผ่นทำความสะอาดครัว ทิชชู่เปียกทำความสะอาด ขจัดคราบน้ำมัน 99% ล้างคราบง่าย</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1Le6P5v0sE</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81zti-mjqfof7pi3nme2.webp</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>฿157.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>128</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>PRO ผลิตภัณฑ์ ล้างจาน โปร ผสมน้ำมะนาว 3,200 ml.</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/BS90x87HP</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztd-mkhuf2c7qqklb6.webp</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>฿125.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>129</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Rabito น้ำยาทำความสะอาด คราบมันฝังแน่นห้องครัว น้ำยาขจัดคราบ ห้องครัว ขจัดคราบไขมันในครัว 500มล. C1</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/6VMCYas7N7</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztd-mi9xmv02k4y099.webp</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>฿91.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>130</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>YTL ลูกกลิ้งกำจัดขน เก็บขนและฝุ่น ลูกกลิ้งทำความสะอาด สีชมพู ขจัดขนแมวและขนสุนัข</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/5Aqoy968AX</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/add9868da3414a6048e9b9c0ef70c7e9.webp</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>฿4.00</t>
         </is>
       </c>
     </row>

</xml_diff>